<commit_message>
Make every ODK form text readable: required messages, plain validation messages and spelled-out labels
Field names, choice names, constraints and calculations are unchanged. The
builder VERSION and manifest move to 2026.10.31.
</commit_message>
<xml_diff>
--- a/odk/forms/crop_sown_registry_harvest.xlsx
+++ b/odk/forms/crop_sown_registry_harvest.xlsx
@@ -462,941 +462,961 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>hint</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>constraint</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>constraint_message</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>relevant</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>calculation</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>read_only</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>appearance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>default</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>choice_filter</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>repeat_count</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>required_message</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>farmer_identity</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Farmer Identity</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>farmer_id</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Farmer ID</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>FR- followed by 12 digits, for example FR-123456789012</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>regex(., '^FR-[0-9]{12}$')</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>The Farmer ID must be FR- followed by 12 digits, for example FR-123456789012.</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="1" t="inlineStr">
         <is>
           <t>Enter the Farmer ID.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>fayda_id_entered</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Fayda ID</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>The 16 digit FAN or the 12 digit FIN. Spaces are allowed.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>regex(translate(., ' ', ''), '^([0-9]{12}|[0-9]{16})$')</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>The Fayda ID must be a 16 digit FAN or a 12 digit FIN. Spaces are allowed.</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="1" t="inlineStr">
         <is>
           <t>Enter the Fayda ID.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>fayda_id</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>translate(${fayda_id_entered}, ' ', '')</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>production_season_info</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Production Season</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="1" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>crop_year</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Crop Year</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>. = number(format-date(today(), '%Y'))</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>Only the current crop year is allowed.</t>
         </is>
       </c>
+      <c r="O8" s="1" t="inlineStr">
+        <is>
+          <t>Enter the crop year.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>select_one crop_season</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>production_season</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Production Season</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="O9" s="1" t="inlineStr">
+        <is>
+          <t>Select the production season.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>harvesting</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Harvesting</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="1" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>land_info_id</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Land ID</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="O12" s="1" t="inlineStr">
+        <is>
+          <t>Enter the Land ID.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>select_multiple cluster_status</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>cluster_status_ids</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Cluster / Non Cluster Status</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Cluster Status</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t>Select the cluster status.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>clustered_details</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Clustered Details</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="1" t="inlineStr">
         <is>
           <t>selected(${cluster_status_ids}, 'clustered')</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>cluster_fpc_name</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>FPC Name</t>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Farmer Production Cluster (FPC) Name</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>select_one crop_maturity</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>cluster_crop_maturity_status</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Crop Maturity Status</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>cluster_harvest_date</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Harvest Date</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>Harvest Date cannot be in the future.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>cluster_area_harvested</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Area Harvested (ha)</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="1" t="inlineStr">
         <is>
           <t>Area Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>cluster_qty_harvested</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Quantity Harvested (quintal)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Harvested (quintals)</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="1" t="inlineStr">
         <is>
           <t>Quantity Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>cluster_post_harvest_loss_pct</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Post – Harvest Loss(%)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>Post-Harvest Loss (%)</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 100</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>Post-Harvest Loss must be between 0 and 100%.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>cluster_qty_stored</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Quantity Stored (quintal)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Stored (quintals)</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${cluster_qty_harvested} and (if(${cluster_qty_sold} = '', 0, ${cluster_qty_sold}) + .) &lt;= ${cluster_qty_harvested}</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Quantity Stored cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>cluster_qty_sold</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Quantity Sold (quintal)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Sold (quintals)</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${cluster_qty_harvested} and (if(${cluster_qty_stored} = '', 0, ${cluster_qty_stored}) + .) &lt;= ${cluster_qty_harvested}</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="1" t="inlineStr">
         <is>
           <t>Quantity Sold cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>independant_details</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>Independent Details</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="1" t="inlineStr">
         <is>
           <t>selected(${cluster_status_ids}, 'independent')</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>select_one_from_file crop_name.csv</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>actual_crop_name</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>Actual Crop Name</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>select_one crop_maturity</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>independent_crop_maturity_status</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>Crop Maturity Status</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>independent_harvest_date</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Harvest Date</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>Harvest Date cannot be in the future.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>independent_area_harvested</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>Area Harvested (ha)</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="1" t="inlineStr">
         <is>
           <t>Area Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>independent_qty_harvested</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Quantity Harvested (quintal)</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Harvested (quintals)</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>Quantity Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>independent_post_harvest_loss_pct</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Post – Harvest Loss(%)</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>Post-Harvest Loss (%)</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 100</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>Post-Harvest Loss must be between 0 and 100%.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>independent_qty_stored</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Quantity Stored (quintal)</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Stored (quintals)</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${independent_qty_harvested} and (if(${independent_qty_sold} = '', 0, ${independent_qty_sold}) + .) &lt;= ${independent_qty_harvested}</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>Quantity Stored cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>independent_qty_sold</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Quantity Sold (quintal)</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Sold (quintals)</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${independent_qty_harvested} and (if(${independent_qty_stored} = '', 0, ${independent_qty_stored}) + .) &lt;= ${independent_qty_harvested}</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="1" t="inlineStr">
         <is>
           <t>Quantity Sold cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>surveyor_name</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>DA Name</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>Development Agent Name</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>regex(., '^[a-zA-Z\u1200-\u137F .\-]+$')</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>DA Name may contain only letters (English or Amharic), spaces, dots and hyphens</t>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>Enter the Development Agent's name using letters (English or Amharic), spaces, dots and hyphens only.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t>surveyor_mobile_number</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>DA Mobile Number</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Format: 0911223344 or +251911223344</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>Development Agent Mobile Number</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>For example 0911223344 or +251911223344</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t>regex(., '^(\+251[79][0-9]{8}|0[79][0-9]{8})$')</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="1" t="inlineStr">
         <is>
           <t>supervisor_name</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="1" t="inlineStr">
         <is>
           <t>Supervisor Name</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="1" t="inlineStr">
         <is>
           <t>regex(., '^[a-zA-Z\u1200-\u137F .\-]+$')</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Supervisor Name may contain only letters (English or Amharic), spaces, dots and hyphens</t>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>Enter the supervisor's name using letters (English or Amharic), spaces, dots and hyphens only.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="1" t="inlineStr">
         <is>
           <t>supervisor_mobile_number</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="1" t="inlineStr">
         <is>
           <t>Supervisor Mobile Number</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Format: 0911223344 or +251911223344</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>For example 0911223344 or +251911223344</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
         <is>
           <t>regex(., '^(\+251[79][0-9]{8}|0[79][0-9]{8})$')</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>end_repeat</t>
         </is>
@@ -1417,136 +1437,136 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>crop_maturity</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>not_yet_ready</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Not Yet Ready</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>crop_maturity</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>ready_for_harvest</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Ready for Harvest</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>cluster_status</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>clustered</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Clustered</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>cluster_status</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>independent</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>SEASON_MEHER</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Meher (main rains)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>SEASON_BELG</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Belg (short rains)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>SEASON_IRRIGATION</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Irrigation (dry season)</t>
         </is>
@@ -1567,64 +1587,64 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>form_title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>form_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>default_language</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>style</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>allow_choice_duplicates</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CSR – 4. Harvesting</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Crop Sown Registry - 4. Harvesting</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>crop_sown_registry_harvest</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026.10.30</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>2026.10.31</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>English (en)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>pages</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
Make every ODK form text readable: required messages, plain validation messages and spelled-out labels (#182)
Field names, choice names, constraints and calculations are unchanged. The
builder VERSION and manifest move to 2026.10.31.
</commit_message>
<xml_diff>
--- a/odk/forms/crop_sown_registry_harvest.xlsx
+++ b/odk/forms/crop_sown_registry_harvest.xlsx
@@ -462,941 +462,961 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>hint</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>constraint</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>constraint_message</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>relevant</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>calculation</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>read_only</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>appearance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>default</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>choice_filter</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>repeat_count</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>required_message</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>farmer_identity</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Farmer Identity</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>farmer_id</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Farmer ID</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>FR- followed by 12 digits, for example FR-123456789012</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>regex(., '^FR-[0-9]{12}$')</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>The Farmer ID must be FR- followed by 12 digits, for example FR-123456789012.</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="1" t="inlineStr">
         <is>
           <t>Enter the Farmer ID.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>fayda_id_entered</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Fayda ID</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>The 16 digit FAN or the 12 digit FIN. Spaces are allowed.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>regex(translate(., ' ', ''), '^([0-9]{12}|[0-9]{16})$')</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>The Fayda ID must be a 16 digit FAN or a 12 digit FIN. Spaces are allowed.</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="1" t="inlineStr">
         <is>
           <t>Enter the Fayda ID.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>fayda_id</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>translate(${fayda_id_entered}, ' ', '')</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>production_season_info</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Production Season</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="1" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>crop_year</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Crop Year</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>. = number(format-date(today(), '%Y'))</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>Only the current crop year is allowed.</t>
         </is>
       </c>
+      <c r="O8" s="1" t="inlineStr">
+        <is>
+          <t>Enter the crop year.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>select_one crop_season</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>production_season</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Production Season</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="O9" s="1" t="inlineStr">
+        <is>
+          <t>Select the production season.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>harvesting</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Harvesting</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="1" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>land_info_id</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Land ID</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="O12" s="1" t="inlineStr">
+        <is>
+          <t>Enter the Land ID.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>select_multiple cluster_status</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>cluster_status_ids</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Cluster / Non Cluster Status</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Cluster Status</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t>Select the cluster status.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>clustered_details</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Clustered Details</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="1" t="inlineStr">
         <is>
           <t>selected(${cluster_status_ids}, 'clustered')</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>cluster_fpc_name</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>FPC Name</t>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Farmer Production Cluster (FPC) Name</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>select_one crop_maturity</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>cluster_crop_maturity_status</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Crop Maturity Status</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>cluster_harvest_date</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Harvest Date</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>Harvest Date cannot be in the future.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>cluster_area_harvested</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Area Harvested (ha)</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="1" t="inlineStr">
         <is>
           <t>Area Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>cluster_qty_harvested</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Quantity Harvested (quintal)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Harvested (quintals)</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="1" t="inlineStr">
         <is>
           <t>Quantity Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>cluster_post_harvest_loss_pct</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Post – Harvest Loss(%)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>Post-Harvest Loss (%)</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 100</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>Post-Harvest Loss must be between 0 and 100%.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>cluster_qty_stored</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Quantity Stored (quintal)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Stored (quintals)</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${cluster_qty_harvested} and (if(${cluster_qty_sold} = '', 0, ${cluster_qty_sold}) + .) &lt;= ${cluster_qty_harvested}</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Quantity Stored cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>cluster_qty_sold</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Quantity Sold (quintal)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Sold (quintals)</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${cluster_qty_harvested} and (if(${cluster_qty_stored} = '', 0, ${cluster_qty_stored}) + .) &lt;= ${cluster_qty_harvested}</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="1" t="inlineStr">
         <is>
           <t>Quantity Sold cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>independant_details</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>Independent Details</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="1" t="inlineStr">
         <is>
           <t>selected(${cluster_status_ids}, 'independent')</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>select_one_from_file crop_name.csv</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>actual_crop_name</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>Actual Crop Name</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>select_one crop_maturity</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>independent_crop_maturity_status</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>Crop Maturity Status</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="1" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>independent_harvest_date</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Harvest Date</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>Harvest Date cannot be in the future.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>independent_area_harvested</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>Area Harvested (ha)</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="1" t="inlineStr">
         <is>
           <t>Area Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>independent_qty_harvested</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Quantity Harvested (quintal)</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Harvested (quintals)</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>Quantity Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>independent_post_harvest_loss_pct</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Post – Harvest Loss(%)</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>Post-Harvest Loss (%)</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 100</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>Post-Harvest Loss must be between 0 and 100%.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>independent_qty_stored</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Quantity Stored (quintal)</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Stored (quintals)</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${independent_qty_harvested} and (if(${independent_qty_sold} = '', 0, ${independent_qty_sold}) + .) &lt;= ${independent_qty_harvested}</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>Quantity Stored cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>independent_qty_sold</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Quantity Sold (quintal)</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Quantity Sold (quintals)</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${independent_qty_harvested} and (if(${independent_qty_stored} = '', 0, ${independent_qty_stored}) + .) &lt;= ${independent_qty_harvested}</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="1" t="inlineStr">
         <is>
           <t>Quantity Sold cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>surveyor_name</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>DA Name</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>Development Agent Name</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>regex(., '^[a-zA-Z\u1200-\u137F .\-]+$')</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>DA Name may contain only letters (English or Amharic), spaces, dots and hyphens</t>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>Enter the Development Agent's name using letters (English or Amharic), spaces, dots and hyphens only.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t>surveyor_mobile_number</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>DA Mobile Number</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Format: 0911223344 or +251911223344</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>Development Agent Mobile Number</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>For example 0911223344 or +251911223344</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t>regex(., '^(\+251[79][0-9]{8}|0[79][0-9]{8})$')</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="1" t="inlineStr">
         <is>
           <t>supervisor_name</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="1" t="inlineStr">
         <is>
           <t>Supervisor Name</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="1" t="inlineStr">
         <is>
           <t>regex(., '^[a-zA-Z\u1200-\u137F .\-]+$')</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Supervisor Name may contain only letters (English or Amharic), spaces, dots and hyphens</t>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>Enter the supervisor's name using letters (English or Amharic), spaces, dots and hyphens only.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="1" t="inlineStr">
         <is>
           <t>supervisor_mobile_number</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="1" t="inlineStr">
         <is>
           <t>Supervisor Mobile Number</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Format: 0911223344 or +251911223344</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>For example 0911223344 or +251911223344</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
         <is>
           <t>regex(., '^(\+251[79][0-9]{8}|0[79][0-9]{8})$')</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>end_repeat</t>
         </is>
@@ -1417,136 +1437,136 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>crop_maturity</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>not_yet_ready</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Not Yet Ready</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>crop_maturity</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>ready_for_harvest</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Ready for Harvest</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>cluster_status</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>clustered</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Clustered</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>cluster_status</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>independent</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>SEASON_MEHER</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Meher (main rains)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>SEASON_BELG</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Belg (short rains)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>SEASON_IRRIGATION</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Irrigation (dry season)</t>
         </is>
@@ -1567,64 +1587,64 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>form_title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>form_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>default_language</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>style</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>allow_choice_duplicates</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CSR – 4. Harvesting</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Crop Sown Registry - 4. Harvesting</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>crop_sown_registry_harvest</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026.10.30</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>2026.10.31</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>English (en)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>pages</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
Crop Sown planning and cultivation: one Variety dropdown
The planning and cultivation tables carried two dropdowns for the planted
variety: Crop Variety (CROP_VARIETY, a Master Data list that is not in
openg2p-data) and Seed Variety (SEED_VARIETY, from the ETH-OAN pack). The
Crop Variety column is removed from both table sections in the base seed and
by a new zz-oan overlay that repairs databases that already hold it, and the
remaining dropdown is labelled Variety (English translations included).

The crop_variety database columns and models are unchanged. The attribute
message list, the CROP_VARIETY prefix handling, the ODK, DCI and file-import
templates, the import template headers and the file-import guide no longer
mention it. The ODK form builder no longer reads or needs CROP_VARIETY: the
Crop Variety question is dropped, the variety question is labelled Variety,
the forms are rebuilt with version 2026.10.31.2 and the CROP_VARIETY export
and crop_variety.csv are deleted.
</commit_message>
<xml_diff>
--- a/odk/forms/crop_sown_registry_harvest.xlsx
+++ b/odk/forms/crop_sown_registry_harvest.xlsx
@@ -192,7 +192,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -251,6 +251,85 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -462,961 +541,961 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>hint</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>constraint</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>constraint_message</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>relevant</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>calculation</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>read_only</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>appearance</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>default</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>choice_filter</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>repeat_count</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>required_message</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>farmer_identity</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Farmer Identity</t>
         </is>
       </c>
-      <c r="K2" s="1" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>farmer_id</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Farmer ID</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>FR- followed by 12 digits, for example FR-123456789012</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>regex(., '^FR-[0-9]{12}$')</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>The Farmer ID must be FR- followed by 12 digits, for example FR-123456789012.</t>
         </is>
       </c>
-      <c r="O3" s="1" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Enter the Farmer ID.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>fayda_id_entered</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Fayda ID</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>The 16 digit FAN or the 12 digit FIN. Spaces are allowed.</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>regex(translate(., ' ', ''), '^([0-9]{12}|[0-9]{16})$')</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>The Fayda ID must be a 16 digit FAN or a 12 digit FIN. Spaces are allowed.</t>
         </is>
       </c>
-      <c r="O4" s="1" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Enter the Fayda ID.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>fayda_id</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>translate(${fayda_id_entered}, ' ', '')</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>production_season_info</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Production Season</t>
         </is>
       </c>
-      <c r="K7" s="1" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>crop_year</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Crop Year</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>. = number(format-date(today(), '%Y'))</t>
         </is>
       </c>
-      <c r="G8" s="1" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Only the current crop year is allowed.</t>
         </is>
       </c>
-      <c r="O8" s="1" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Enter the crop year.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>select_one crop_season</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>production_season</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Production Season</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="O9" s="1" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Select the production season.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>harvesting</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Harvesting</t>
         </is>
       </c>
-      <c r="K11" s="1" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>land_info_id</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Land ID</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="O12" s="1" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Enter the Land ID.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>select_multiple cluster_status</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>cluster_status_ids</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Cluster Status</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K13" s="1" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
-      <c r="O13" s="1" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Select the cluster status.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>clustered_details</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Clustered Details</t>
         </is>
       </c>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>selected(${cluster_status_ids}, 'clustered')</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>cluster_fpc_name</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Farmer Production Cluster (FPC) Name</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>select_one crop_maturity</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>cluster_crop_maturity_status</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Crop Maturity Status</t>
         </is>
       </c>
-      <c r="K16" s="1" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>cluster_harvest_date</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Harvest Date</t>
         </is>
       </c>
-      <c r="G17" s="1" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Harvest Date cannot be in the future.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>cluster_area_harvested</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Area Harvested (ha)</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G18" s="1" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Area Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>cluster_qty_harvested</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Quantity Harvested (quintals)</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G19" s="1" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Quantity Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>cluster_post_harvest_loss_pct</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Post-Harvest Loss (%)</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 100</t>
         </is>
       </c>
-      <c r="G20" s="1" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Post-Harvest Loss must be between 0 and 100%.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>cluster_qty_stored</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Quantity Stored (quintals)</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${cluster_qty_harvested} and (if(${cluster_qty_sold} = '', 0, ${cluster_qty_sold}) + .) &lt;= ${cluster_qty_harvested}</t>
         </is>
       </c>
-      <c r="G21" s="1" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Quantity Stored cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>cluster_qty_sold</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Quantity Sold (quintals)</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${cluster_qty_harvested} and (if(${cluster_qty_stored} = '', 0, ${cluster_qty_stored}) + .) &lt;= ${cluster_qty_harvested}</t>
         </is>
       </c>
-      <c r="G22" s="1" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Quantity Sold cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>independant_details</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Independent Details</t>
         </is>
       </c>
-      <c r="H24" s="1" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>selected(${cluster_status_ids}, 'independent')</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>select_one_from_file crop_name.csv</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>actual_crop_name</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Actual Crop Name</t>
         </is>
       </c>
-      <c r="K25" s="1" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>select_one crop_maturity</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>independent_crop_maturity_status</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Crop Maturity Status</t>
         </is>
       </c>
-      <c r="K26" s="1" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>independent_harvest_date</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Harvest Date</t>
         </is>
       </c>
-      <c r="G27" s="1" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Harvest Date cannot be in the future.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>independent_area_harvested</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Area Harvested (ha)</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G28" s="1" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Area Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>independent_qty_harvested</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Quantity Harvested (quintals)</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>. &gt; 0</t>
         </is>
       </c>
-      <c r="G29" s="1" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Quantity Harvested must be greater than 0.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>independent_post_harvest_loss_pct</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Post-Harvest Loss (%)</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 100</t>
         </is>
       </c>
-      <c r="G30" s="1" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Post-Harvest Loss must be between 0 and 100%.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>independent_qty_stored</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Quantity Stored (quintals)</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${independent_qty_harvested} and (if(${independent_qty_sold} = '', 0, ${independent_qty_sold}) + .) &lt;= ${independent_qty_harvested}</t>
         </is>
       </c>
-      <c r="G31" s="1" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Quantity Stored cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>decimal</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>independent_qty_sold</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Quantity Sold (quintals)</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= ${independent_qty_harvested} and (if(${independent_qty_stored} = '', 0, ${independent_qty_stored}) + .) &lt;= ${independent_qty_harvested}</t>
         </is>
       </c>
-      <c r="G32" s="1" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Quantity Sold cannot be negative, and Stored + Sold cannot exceed Quantity Harvested.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>surveyor_name</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Development Agent Name</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>regex(., '^[a-zA-Z\u1200-\u137F .\-]+$')</t>
         </is>
       </c>
-      <c r="G34" s="1" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Enter the Development Agent's name using letters (English or Amharic), spaces, dots and hyphens only.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>surveyor_mobile_number</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Development Agent Mobile Number</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>For example 0911223344 or +251911223344</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>regex(., '^(\+251[79][0-9]{8}|0[79][0-9]{8})$')</t>
         </is>
       </c>
-      <c r="G35" s="1" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B36" s="1" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>supervisor_name</t>
         </is>
       </c>
-      <c r="C36" s="1" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Supervisor Name</t>
         </is>
       </c>
-      <c r="F36" s="1" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>regex(., '^[a-zA-Z\u1200-\u137F .\-]+$')</t>
         </is>
       </c>
-      <c r="G36" s="1" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Enter the supervisor's name using letters (English or Amharic), spaces, dots and hyphens only.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B37" s="1" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>supervisor_mobile_number</t>
         </is>
       </c>
-      <c r="C37" s="1" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Supervisor Mobile Number</t>
         </is>
       </c>
-      <c r="D37" s="1" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>For example 0911223344 or +251911223344</t>
         </is>
       </c>
-      <c r="F37" s="1" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>regex(., '^(\+251[79][0-9]{8}|0[79][0-9]{8})$')</t>
         </is>
       </c>
-      <c r="G37" s="1" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>end_repeat</t>
         </is>
@@ -1437,136 +1516,136 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>crop_maturity</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>not_yet_ready</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Not Yet Ready</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>crop_maturity</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>ready_for_harvest</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Ready for Harvest</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>cluster_status</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>clustered</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Clustered</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>cluster_status</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>independent</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>SEASON_MEHER</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Meher (main rains)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>SEASON_BELG</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Belg (short rains)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>crop_season</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>SEASON_IRRIGATION</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Irrigation (dry season)</t>
         </is>
@@ -1587,64 +1666,64 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>form_title</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>form_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>default_language</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>style</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>allow_choice_duplicates</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Crop Sown Registry - 4. Harvesting</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>crop_sown_registry_harvest</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>2026.10.31.1</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026.10.31.2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>English (en)</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>pages</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>